<commit_message>
png not break anymore, but site label still broken
</commit_message>
<xml_diff>
--- a/5-png-inserter/out/test_fixture.xlsx
+++ b/5-png-inserter/out/test_fixture.xlsx
@@ -233,7 +233,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>49</row>
+      <row>55</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="4762500"/>
@@ -429,7 +429,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>305</row>
+      <row>325</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="5143500"/>
@@ -515,7 +515,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>44</row>
+      <row>55</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="8572500"/>
@@ -543,7 +543,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>92</row>
+      <row>109</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="1781175"/>
@@ -571,7 +571,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>110</row>
+      <row>164</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="3257550"/>
@@ -599,7 +599,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>164</row>
+      <row>218</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="3257550"/>
@@ -627,7 +627,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>218</row>
+      <row>272</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="3257550"/>
@@ -655,7 +655,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>272</row>
+      <row>326</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="1609725"/>
@@ -683,7 +683,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>283</row>
+      <row>337</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="3810000"/>
@@ -711,7 +711,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>306</row>
+      <row>360</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="1038225"/>
@@ -739,7 +739,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>314</row>
+      <row>379</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="2857500" cy="2143125"/>
@@ -1182,7 +1182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K271"/>
+  <dimension ref="A1:K325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1255,29 +1255,29 @@
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="1" t="inlineStr">
-        <is>
-          <t>BKK02</t>
-        </is>
-      </c>
-    </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>BKK03</t>
+          <t>BKK02</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>BKK04</t>
+          <t>BKK03</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
+        <is>
+          <t>BKK04</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="1" t="inlineStr">
         <is>
           <t>BKK09</t>
         </is>
@@ -1287,17 +1287,17 @@
   <mergeCells count="5">
     <mergeCell ref="A163:K163"/>
     <mergeCell ref="A271:K271"/>
-    <mergeCell ref="A109:K109"/>
     <mergeCell ref="A10:K10"/>
     <mergeCell ref="A217:K217"/>
+    <mergeCell ref="A325:K325"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <rowBreaks count="4" manualBreakCount="4">
-    <brk id="109" min="0" max="16383" man="1"/>
     <brk id="163" min="0" max="16383" man="1"/>
     <brk id="217" min="0" max="16383" man="1"/>
     <brk id="271" min="0" max="16383" man="1"/>
+    <brk id="325" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>